<commit_message>
Update dictionaries to include ties to RIInstallationRecord
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/grout_inj_properties.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/grout_inj_properties.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10413"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10726"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dponti/GitHub/def/Codelist Excel Files and Conversion Templates to XML/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dponti/Documents/GitHub/def/Codelist Excel Files and Conversion Templates to XML/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AB35EA3-9C22-FB45-873E-75EEB1A08AC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5557A045-0F2D-F149-8CD2-AB4A31DBCC07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11720" yWindow="3840" windowWidth="35840" windowHeight="20900" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
     <sheet name="AssociatedElements" sheetId="2" r:id="rId3"/>
     <sheet name="Lists" sheetId="5" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="348">
   <si>
     <t>Description</t>
   </si>
@@ -992,9 +992,6 @@
     <t>pull_speed</t>
   </si>
   <si>
-    <t>pull speed</t>
-  </si>
-  <si>
     <t>Lift rate of the monitor while grouting</t>
   </si>
   <si>
@@ -1077,13 +1074,19 @@
   </si>
   <si>
     <t>ancestor::diggs:ContinuousGrouting</t>
+  </si>
+  <si>
+    <t>pull speed|withdrawal rate</t>
+  </si>
+  <si>
+    <t>ancestor::diggs:constructionActivity//diggs:RIInstallationRecord</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1187,6 +1190,12 @@
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Helvetica"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -1299,7 +1308,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1345,16 +1354,21 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
@@ -1370,77 +1384,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="22">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <color theme="0"/>
-      </font>
-    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1579,6 +1522,77 @@
       </font>
       <alignment horizontal="general" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="0"/>
+      </font>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium7"/>
   <extLst>
@@ -1593,51 +1607,51 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="DictionaryName" displayName="DictionaryName" ref="A1:E3" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="DictionaryName" displayName="DictionaryName" ref="A1:E3" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
   <autoFilter ref="A1:E3" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Start" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Dictionary ID" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="DictionaryFile" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="DictionaryName" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Description" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Start" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Dictionary ID" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="DictionaryFile" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="DictionaryName" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Description" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Definitions" displayName="Definitions" ref="A1:H37" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Definitions" displayName="Definitions" ref="A1:H37" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
   <autoFilter ref="A1:H37" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Start" dataDxfId="12">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Start" dataDxfId="7">
       <calculatedColumnFormula>IF(ISNA(VLOOKUP(B2,AssociatedElements!B$2:B872,1,FALSE)),"Not used","")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="ID" dataDxfId="11"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Name" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Description" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="DataType" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="QuantityClass" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Authority" dataDxfId="6"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="Reference" dataDxfId="5"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="ID" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Name" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Description" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="DataType" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="QuantityClass" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Authority" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="Reference" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="AssociatedElements" displayName="AssociatedElements" ref="A1:E45" totalsRowShown="0" headerRowDxfId="4">
-  <autoFilter ref="A1:E45" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C2">
-    <sortCondition ref="C1:C2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="AssociatedElements" displayName="AssociatedElements" ref="A1:E48" totalsRowShown="0" headerRowDxfId="21">
+  <autoFilter ref="A1:E48" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E45">
+    <sortCondition ref="B1:B45"/>
   </sortState>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Start" dataDxfId="3">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Start" dataDxfId="20">
       <calculatedColumnFormula>IF(ISNA(VLOOKUP(B2,Definitions!B$2:B$1843,1,FALSE)),"Not listed","")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="ID" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="SourceElement" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="ConditionalElement" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="ID" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="SourceElement" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="ConditionalElement" dataDxfId="17"/>
     <tableColumn id="5" xr3:uid="{70DA9ABB-01EE-9C4D-9F26-0BFC80A8CC6E}" name="Column1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1962,7 +1976,7 @@
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" ht="51" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>233</v>
@@ -1971,7 +1985,7 @@
         <v>234</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
   </sheetData>
@@ -2630,10 +2644,10 @@
         <v>317</v>
       </c>
       <c r="C29" s="17" t="s">
+        <v>346</v>
+      </c>
+      <c r="D29" s="17" t="s">
         <v>318</v>
-      </c>
-      <c r="D29" s="17" t="s">
-        <v>319</v>
       </c>
       <c r="E29" s="19" t="s">
         <v>1</v>
@@ -2649,13 +2663,13 @@
         <v/>
       </c>
       <c r="B30" s="16" t="s">
+        <v>319</v>
+      </c>
+      <c r="C30" s="17" t="s">
         <v>320</v>
       </c>
-      <c r="C30" s="17" t="s">
+      <c r="D30" s="17" t="s">
         <v>321</v>
-      </c>
-      <c r="D30" s="17" t="s">
-        <v>322</v>
       </c>
       <c r="E30" s="19" t="s">
         <v>1</v>
@@ -2671,13 +2685,13 @@
         <v/>
       </c>
       <c r="B31" s="16" t="s">
+        <v>322</v>
+      </c>
+      <c r="C31" s="17" t="s">
         <v>323</v>
       </c>
-      <c r="C31" s="17" t="s">
+      <c r="D31" s="17" t="s">
         <v>324</v>
-      </c>
-      <c r="D31" s="17" t="s">
-        <v>325</v>
       </c>
       <c r="E31" s="19" t="s">
         <v>1</v>
@@ -2693,19 +2707,19 @@
         <v/>
       </c>
       <c r="B32" s="16" t="s">
+        <v>325</v>
+      </c>
+      <c r="C32" s="17" t="s">
         <v>326</v>
       </c>
-      <c r="C32" s="17" t="s">
+      <c r="D32" s="17" t="s">
         <v>327</v>
-      </c>
-      <c r="D32" s="17" t="s">
-        <v>328</v>
       </c>
       <c r="E32" s="19" t="s">
         <v>1</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="G32" s="11"/>
     </row>
@@ -2715,13 +2729,13 @@
         <v/>
       </c>
       <c r="B33" s="16" t="s">
+        <v>329</v>
+      </c>
+      <c r="C33" s="17" t="s">
         <v>330</v>
       </c>
-      <c r="C33" s="17" t="s">
+      <c r="D33" s="17" t="s">
         <v>331</v>
-      </c>
-      <c r="D33" s="17" t="s">
-        <v>332</v>
       </c>
       <c r="E33" s="19" t="s">
         <v>180</v>
@@ -2737,13 +2751,13 @@
         <v/>
       </c>
       <c r="B34" s="16" t="s">
+        <v>332</v>
+      </c>
+      <c r="C34" s="17" t="s">
         <v>333</v>
       </c>
-      <c r="C34" s="17" t="s">
+      <c r="D34" s="17" t="s">
         <v>334</v>
-      </c>
-      <c r="D34" s="17" t="s">
-        <v>335</v>
       </c>
       <c r="E34" s="19" t="s">
         <v>1</v>
@@ -2759,13 +2773,13 @@
         <v/>
       </c>
       <c r="B35" s="16" t="s">
+        <v>335</v>
+      </c>
+      <c r="C35" s="17" t="s">
+        <v>335</v>
+      </c>
+      <c r="D35" s="17" t="s">
         <v>336</v>
-      </c>
-      <c r="C35" s="17" t="s">
-        <v>336</v>
-      </c>
-      <c r="D35" s="17" t="s">
-        <v>337</v>
       </c>
       <c r="E35" s="19" t="s">
         <v>1</v>
@@ -2781,13 +2795,13 @@
         <v/>
       </c>
       <c r="B36" s="16" t="s">
+        <v>337</v>
+      </c>
+      <c r="C36" s="18" t="s">
+        <v>337</v>
+      </c>
+      <c r="D36" s="18" t="s">
         <v>338</v>
-      </c>
-      <c r="C36" s="18" t="s">
-        <v>338</v>
-      </c>
-      <c r="D36" s="18" t="s">
-        <v>339</v>
       </c>
       <c r="E36" s="19" t="s">
         <v>1</v>
@@ -2808,13 +2822,13 @@
       <c r="C37" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="D37" s="23" t="s">
-        <v>342</v>
-      </c>
-      <c r="E37" s="22" t="s">
+      <c r="D37" s="22" t="s">
+        <v>341</v>
+      </c>
+      <c r="E37" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="F37" s="22" t="s">
+      <c r="F37" s="21" t="s">
         <v>25</v>
       </c>
       <c r="G37" s="11"/>
@@ -2843,7 +2857,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
@@ -2866,7 +2880,7 @@
         <v>226</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -2877,11 +2891,11 @@
       <c r="B2" s="14" t="s">
         <v>235</v>
       </c>
-      <c r="C2" s="24" t="s">
+      <c r="C2" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>344</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -2892,11 +2906,11 @@
       <c r="B3" s="14" t="s">
         <v>238</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="C3" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>344</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -2907,11 +2921,11 @@
       <c r="B4" s="14" t="s">
         <v>241</v>
       </c>
-      <c r="C4" s="24" t="s">
-        <v>344</v>
+      <c r="C4" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -2922,11 +2936,11 @@
       <c r="B5" s="14" t="s">
         <v>244</v>
       </c>
-      <c r="C5" s="24" t="s">
-        <v>344</v>
+      <c r="C5" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -2937,11 +2951,11 @@
       <c r="B6" s="14" t="s">
         <v>246</v>
       </c>
-      <c r="C6" s="24" t="s">
-        <v>344</v>
+      <c r="C6" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -2952,11 +2966,11 @@
       <c r="B7" s="14" t="s">
         <v>249</v>
       </c>
-      <c r="C7" s="24" t="s">
-        <v>344</v>
+      <c r="C7" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -2967,11 +2981,11 @@
       <c r="B8" s="14" t="s">
         <v>252</v>
       </c>
-      <c r="C8" s="24" t="s">
+      <c r="C8" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>344</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -2982,11 +2996,11 @@
       <c r="B9" t="s">
         <v>255</v>
       </c>
-      <c r="C9" s="24" t="s">
+      <c r="C9" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>344</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
@@ -2997,11 +3011,11 @@
       <c r="B10" t="s">
         <v>255</v>
       </c>
-      <c r="C10" s="24" t="s">
-        <v>344</v>
+      <c r="C10" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
@@ -3012,11 +3026,11 @@
       <c r="B11" s="14" t="s">
         <v>258</v>
       </c>
-      <c r="C11" s="24" t="s">
-        <v>344</v>
+      <c r="C11" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
@@ -3027,11 +3041,11 @@
       <c r="B12" s="14" t="s">
         <v>261</v>
       </c>
-      <c r="C12" s="24" t="s">
-        <v>344</v>
+      <c r="C12" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
@@ -3042,11 +3056,11 @@
       <c r="B13" s="14" t="s">
         <v>264</v>
       </c>
-      <c r="C13" s="24" t="s">
-        <v>344</v>
+      <c r="C13" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
@@ -3057,11 +3071,11 @@
       <c r="B14" s="14" t="s">
         <v>267</v>
       </c>
-      <c r="C14" s="24" t="s">
-        <v>344</v>
+      <c r="C14" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
@@ -3072,11 +3086,11 @@
       <c r="B15" s="14" t="s">
         <v>270</v>
       </c>
-      <c r="C15" s="24" t="s">
-        <v>344</v>
+      <c r="C15" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
@@ -3087,11 +3101,11 @@
       <c r="B16" s="14" t="s">
         <v>273</v>
       </c>
-      <c r="C16" s="24" t="s">
-        <v>344</v>
+      <c r="C16" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
@@ -3102,11 +3116,11 @@
       <c r="B17" s="14" t="s">
         <v>276</v>
       </c>
-      <c r="C17" s="24" t="s">
-        <v>344</v>
+      <c r="C17" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
@@ -3117,11 +3131,11 @@
       <c r="B18" s="14" t="s">
         <v>279</v>
       </c>
-      <c r="C18" s="24" t="s">
+      <c r="C18" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="D18" s="3" t="s">
         <v>344</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
@@ -3132,11 +3146,11 @@
       <c r="B19" s="14" t="s">
         <v>279</v>
       </c>
-      <c r="C19" s="24" t="s">
-        <v>344</v>
+      <c r="C19" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
@@ -3147,11 +3161,11 @@
       <c r="B20" s="14" t="s">
         <v>282</v>
       </c>
-      <c r="C20" s="24" t="s">
+      <c r="C20" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="D20" s="3" t="s">
         <v>344</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
@@ -3162,11 +3176,11 @@
       <c r="B21" s="14" t="s">
         <v>282</v>
       </c>
-      <c r="C21" s="24" t="s">
-        <v>344</v>
+      <c r="C21" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
@@ -3177,11 +3191,11 @@
       <c r="B22" s="14" t="s">
         <v>285</v>
       </c>
-      <c r="C22" s="24" t="s">
+      <c r="C22" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="D22" s="3" t="s">
         <v>344</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
@@ -3192,11 +3206,11 @@
       <c r="B23" s="14" t="s">
         <v>285</v>
       </c>
-      <c r="C23" s="24" t="s">
-        <v>344</v>
+      <c r="C23" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
@@ -3207,11 +3221,11 @@
       <c r="B24" s="14" t="s">
         <v>288</v>
       </c>
-      <c r="C24" s="24" t="s">
+      <c r="C24" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="D24" s="3" t="s">
         <v>344</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
@@ -3222,11 +3236,11 @@
       <c r="B25" s="14" t="s">
         <v>288</v>
       </c>
-      <c r="C25" s="24" t="s">
-        <v>344</v>
+      <c r="C25" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
@@ -3237,11 +3251,11 @@
       <c r="B26" s="14" t="s">
         <v>291</v>
       </c>
-      <c r="C26" s="24" t="s">
-        <v>344</v>
+      <c r="C26" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
@@ -3252,11 +3266,11 @@
       <c r="B27" s="14" t="s">
         <v>294</v>
       </c>
-      <c r="C27" s="24" t="s">
-        <v>344</v>
+      <c r="C27" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
@@ -3267,11 +3281,11 @@
       <c r="B28" s="14" t="s">
         <v>297</v>
       </c>
-      <c r="C28" s="24" t="s">
+      <c r="C28" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="D28" s="3" t="s">
         <v>344</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
@@ -3282,11 +3296,11 @@
       <c r="B29" s="14" t="s">
         <v>300</v>
       </c>
-      <c r="C29" s="24" t="s">
+      <c r="C29" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="D29" t="s">
         <v>344</v>
-      </c>
-      <c r="D29" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
@@ -3297,11 +3311,11 @@
       <c r="B30" s="14" t="s">
         <v>304</v>
       </c>
-      <c r="C30" s="24" t="s">
-        <v>344</v>
+      <c r="C30" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
@@ -3312,11 +3326,11 @@
       <c r="B31" s="14" t="s">
         <v>307</v>
       </c>
-      <c r="C31" s="24" t="s">
-        <v>344</v>
+      <c r="C31" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
@@ -3327,11 +3341,11 @@
       <c r="B32" s="14" t="s">
         <v>310</v>
       </c>
-      <c r="C32" s="24" t="s">
+      <c r="C32" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="D32" t="s">
         <v>344</v>
-      </c>
-      <c r="D32" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
@@ -3342,11 +3356,11 @@
       <c r="B33" s="14" t="s">
         <v>314</v>
       </c>
-      <c r="C33" s="24" t="s">
+      <c r="C33" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="D33" t="s">
         <v>344</v>
-      </c>
-      <c r="D33" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
@@ -3357,11 +3371,11 @@
       <c r="B34" s="14" t="s">
         <v>317</v>
       </c>
-      <c r="C34" s="24" t="s">
-        <v>344</v>
+      <c r="C34" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
@@ -3370,13 +3384,13 @@
         <v/>
       </c>
       <c r="B35" s="14" t="s">
-        <v>320</v>
-      </c>
-      <c r="C35" s="24" t="s">
-        <v>344</v>
+        <v>319</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
@@ -3385,13 +3399,13 @@
         <v/>
       </c>
       <c r="B36" s="14" t="s">
-        <v>323</v>
-      </c>
-      <c r="C36" s="24" t="s">
-        <v>344</v>
+        <v>322</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
@@ -3400,13 +3414,13 @@
         <v/>
       </c>
       <c r="B37" s="14" t="s">
-        <v>326</v>
-      </c>
-      <c r="C37" s="24" t="s">
-        <v>344</v>
+        <v>325</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
@@ -3415,13 +3429,13 @@
         <v/>
       </c>
       <c r="B38" s="14" t="s">
-        <v>330</v>
-      </c>
-      <c r="C38" s="24" t="s">
-        <v>344</v>
+        <v>329</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
@@ -3430,13 +3444,13 @@
         <v/>
       </c>
       <c r="B39" t="s">
-        <v>330</v>
-      </c>
-      <c r="C39" s="24" t="s">
-        <v>344</v>
+        <v>329</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
@@ -3445,13 +3459,13 @@
         <v/>
       </c>
       <c r="B40" t="s">
-        <v>333</v>
-      </c>
-      <c r="C40" s="24" t="s">
+        <v>332</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="D40" s="20" t="s">
         <v>344</v>
-      </c>
-      <c r="D40" s="20" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
@@ -3460,13 +3474,13 @@
         <v/>
       </c>
       <c r="B41" t="s">
-        <v>333</v>
-      </c>
-      <c r="C41" s="24" t="s">
-        <v>344</v>
+        <v>332</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
@@ -3475,13 +3489,13 @@
         <v/>
       </c>
       <c r="B42" s="14" t="s">
-        <v>336</v>
-      </c>
-      <c r="C42" s="24" t="s">
-        <v>344</v>
+        <v>335</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
@@ -3490,14 +3504,15 @@
         <v/>
       </c>
       <c r="B43" s="14" t="s">
-        <v>338</v>
-      </c>
-      <c r="C43" s="24" t="s">
-        <v>344</v>
+        <v>25</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>346</v>
-      </c>
+        <v>345</v>
+      </c>
+      <c r="E43" s="23"/>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44" t="str">
@@ -3507,13 +3522,13 @@
       <c r="B44" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="C44" s="24" t="s">
+      <c r="C44" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="D44" s="3" t="s">
         <v>344</v>
       </c>
-      <c r="D44" s="3" t="s">
-        <v>346</v>
-      </c>
-      <c r="E44" s="21"/>
+      <c r="E44" s="24"/>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45" t="str">
@@ -3521,13 +3536,58 @@
         <v/>
       </c>
       <c r="B45" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="C45" s="24" t="s">
-        <v>344</v>
+        <v>337</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="D45" s="3" t="s">
         <v>345</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A46" s="25" t="str">
+        <f>IF(ISNA(VLOOKUP(B46,Definitions!B$2:B$1843,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B46" s="26" t="s">
+        <v>317</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="D46" s="27" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A47" s="25" t="str">
+        <f>IF(ISNA(VLOOKUP(B47,Definitions!B$2:B$1843,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B47" s="26" t="s">
+        <v>282</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="D47" s="27" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A48" s="25" t="str">
+        <f>IF(ISNA(VLOOKUP(B48,Definitions!B$2:B$1843,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B48" s="26" t="s">
+        <v>279</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="D48" s="27" t="s">
+        <v>347</v>
       </c>
     </row>
   </sheetData>

</xml_diff>